<commit_message>
Aggiorna tariffe orarie reali nel team
Senior Graphic Designer: €15/h
Junior Graphic Designer: €8/h
Video Editor: €8/h

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_team_data.xlsx
+++ b/ai_team_data.xlsx
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -1058,7 +1058,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -1120,7 +1120,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1316,9 +1316,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1333,9 +1331,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -1392,9 +1388,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
@@ -1451,9 +1445,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
@@ -1489,9 +1481,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-    </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
@@ -1534,9 +1524,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-    </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
@@ -1558,9 +1546,7 @@
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-    </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Refactor completo: minuti/unità editabili, labels in giorni, task generici
Logica:
- Sostituito asset_per_giorno con minuti_per_unita (editabile per progetto in UI)
- Ore = (quantità × min/unità) / 60 × overhead
- Output in ore e giorni lavorativi (no MD, no settimane)
- Durata calendario in giorni lun-ven

Excel:
- Nomi lavorazioni generici (rimosso Qatar, cliente moda)
- Rimossa categoria EDITING
- Martina Lorini e Anna Zonca → Junior Graphic Designer

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_team_data.xlsx
+++ b/ai_team_data.xlsx
@@ -183,46 +183,6 @@
 </file>
 
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>AI_Team</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>ID univoco. Convenzione: VID-GS-01 = VIDEO / GENERAZIONE STATICI / n. 01.</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>Macro-categoria. Per estendere: aggiungi STATICI, PDP, ecc.</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>Raggruppamento dentro la categoria. Usato per organizzare la UI.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Distinzione fine tra versioni della stessa lavorazione (es. Qatar vs cliente moda).</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Quanti asset completi produce 1 risorsa in una giornata standard da 8h. SOLO numero.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>Una skill per riga. Deve matchare un tag in team.skill_tags.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>AI_Team</author>
@@ -551,373 +511,283 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tipologia_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>sottocategoria</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>nome_lavorazione</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>variante</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>asset_per_giorno</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>minuti_per_unita</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>skill_richiesta</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>VID-GS-01</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>VIDEO</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>GENERAZIONE STATICI</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Generazione frame statico in 1 formato</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Qatar</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GS-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GRAFICA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GENERAZIONE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Generazione immagine AI (1 formato)</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>retouch</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>VID-GS-02</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>VIDEO</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>GENERAZIONE STATICI</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Post-produzione generica su frame statico</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>base</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GS-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GRAFICA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GENERAZIONE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Generazione immagine AI (multi-formato)</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>retouch</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>VID-GS-03</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>VIDEO</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>GENERAZIONE STATICI</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GS-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GRAFICA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>POST-PRODUZIONE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Post-produzione base</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>48</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>retouch</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GS-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GRAFICA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>POST-PRODUZIONE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>Post-produzione complessa</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>complessa</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="E5" t="n">
+        <v>240</v>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>retouch</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>VID-AS-01</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>VIDEO</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>ANIMAZIONE STATICI</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Generazione animazione frame statico in 1 formato</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Qatar</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>VID-AS-02</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>VIDEO</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>ANIMAZIONE STATICI</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Generazione animazione frame statico in 1 formato</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>cliente moda</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>VID-AS-03</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>VIDEO</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>ANIMAZIONE STATICI</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Post-produzione base (color)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>color</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GS-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GRAFICA</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ANIMAZIONE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Animazione frame statico (semplice)</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>60</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>retouch</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GS-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GRAFICA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ANIMAZIONE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Animazione frame statico (complessa)</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>120</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>retouch</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GS-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GRAFICA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ANIMAZIONE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Post-produzione animazione (color)</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>40</v>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>compositing</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>VID-AS-04</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>VIDEO</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>ANIMAZIONE STATICI</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Post-produzione con tracking</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>tracking</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GS-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GRAFICA</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ANIMAZIONE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Post-produzione animazione (tracking)</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>160</v>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>compositing</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>VID-ED-01</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>VIDEO</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>EDITING</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Editing base</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>solo messa in fila</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>editing</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>VID-ED-02</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>VIDEO</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>EDITING</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Editing avanzato</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>raccordi, movimenti camera</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>editing</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1235,12 +1105,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Video Editor</t>
+          <t>Junior Graphic Designer</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>junior</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
@@ -1248,7 +1118,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>video,editing,compositing</t>
+          <t>retouch,prompt</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
@@ -1266,12 +1136,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Video Editor</t>
+          <t>Junior Graphic Designer</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>junior</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -1279,7 +1149,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>video,editing,compositing</t>
+          <t>retouch,prompt</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
@@ -1316,7 +1186,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1331,7 +1200,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -1388,7 +1256,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
@@ -1445,7 +1312,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
@@ -1481,7 +1347,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
@@ -1524,7 +1389,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
@@ -1546,7 +1410,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Aggiorna lavorazioni: semplificate, aggiunte color correction e video AI
- Rimossa distinzione base/complessa
- Aggiunta: Color correction foto, Color correction video
- Aggiunta: Generazione video AI
- Lavorazioni VIDEO separate da GRAFICA

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_team_data.xlsx
+++ b/ai_team_data.xlsx
@@ -564,11 +564,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Generazione immagine AI (1 formato)</t>
+          <t>Generazione immagine AI</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>96</v>
+        <v>60</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -589,12 +589,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GENERAZIONE</t>
+          <t>POST-PRODUZIONE</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Generazione immagine AI (multi-formato)</t>
+          <t>Post-produzione immagine</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -619,20 +619,20 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>POST-PRODUZIONE</t>
+          <t>COLOR CORRECTION</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Post-produzione base</t>
+          <t>Color correction foto</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>retouch</t>
+          <t>compositing</t>
         </is>
       </c>
     </row>
@@ -649,16 +649,16 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>POST-PRODUZIONE</t>
+          <t>ANIMAZIONE</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Post-produzione complessa</t>
+          <t>Animazione frame statico</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>240</v>
+        <v>90</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -684,37 +684,37 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Animazione frame statico (semplice)</t>
+          <t>Post-produzione animazione</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>retouch</t>
+          <t>compositing</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GS-06</t>
+          <t>VID-01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GRAFICA</t>
+          <t>VIDEO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ANIMAZIONE</t>
+          <t>GENERAZIONE</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Animazione frame statico (complessa)</t>
+          <t>Generazione video AI</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -722,33 +722,33 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>retouch</t>
+          <t>video</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GS-07</t>
+          <t>VID-02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GRAFICA</t>
+          <t>VIDEO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ANIMAZIONE</t>
+          <t>POST-PRODUZIONE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Post-produzione animazione (color)</t>
+          <t>Post-produzione video</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -759,26 +759,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GS-08</t>
+          <t>VID-03</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GRAFICA</t>
+          <t>VIDEO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ANIMAZIONE</t>
+          <t>COLOR CORRECTION</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Post-produzione animazione (tracking)</t>
+          <t>Color correction video</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>160</v>
+        <v>45</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: add production costs to lavorazioni — Imagen 4 Ultra + Veo 3.1
- Generazione immagine AI: €0.22/unit (NanoBanana Pro 4K / Imagen 4 Ultra)
- Generazione video AI: €3.68/unit (Veo 3.1 4K no audio, 8s clip)
- RETRY_MULTIPLIER=3 already active → effective costs €0.66/img, €11.04/video

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_team_data.xlsx
+++ b/ai_team_data.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,49 +27,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001F2937"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001F2937"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00B91C1C"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F2937"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -77,35 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D1D5DB"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D1D5DB"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D1D5DB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D1D5DB"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -180,46 +124,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>AI_Team</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>ID numerico univoco e stabile. Non riutilizzare se qualcuno esce dal team.</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>Ruolo aziendale (Senior/Junior Graphic Designer, Video Editor, ...). Serve per raggruppamento.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Livello seniority (menu a tendina). Usato per logiche future di allocazione.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Costo orario interno in €. Solo numero, senza simbolo €. VALORI PLACEHOLDER - aggiornare con tariffe reali.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Skill separate da virgola, minuscolo, senza spazi. Devono matchare le skill in 'lavorazioni'.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>Ore realmente allocabili a CM1 a settimana (non il contratto totale).</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -511,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,6 +449,11 @@
           <t>skill_richiesta</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>costo_per_unita_eur</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -575,6 +484,9 @@
           <t>retouch</t>
         </is>
       </c>
+      <c r="G2" t="n">
+        <v>0.22</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -605,6 +517,9 @@
           <t>retouch</t>
         </is>
       </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -635,6 +550,9 @@
           <t>compositing</t>
         </is>
       </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -665,6 +583,9 @@
           <t>retouch</t>
         </is>
       </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -695,6 +616,9 @@
           <t>compositing</t>
         </is>
       </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -725,6 +649,9 @@
           <t>video</t>
         </is>
       </c>
+      <c r="G7" t="n">
+        <v>3.68</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -755,6 +682,9 @@
           <t>compositing</t>
         </is>
       </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -784,6 +714,9 @@
         <is>
           <t>compositing</t>
         </is>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -799,371 +732,356 @@
   </sheetPr>
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>nome</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ruolo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>seniority</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>costo_orario</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>skill_tags</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>disponibilita_h_settimana</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="n">
+    <row r="2">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Manuel Ricciardi</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Senior Graphic Designer</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>senior</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" t="n">
         <v>15</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>retouch,compositing,lighting</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="2" t="n">
+    <row r="3">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Alvar S. Rodriguez</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Senior Graphic Designer</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>senior</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" t="n">
         <v>15</v>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>retouch,compositing,lighting</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="2" t="n">
+    <row r="4">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Elisa Righi</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Senior Graphic Designer</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>senior</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" t="n">
         <v>15</v>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>retouch,compositing,lighting</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="2" t="n">
+    <row r="5">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Andrea Zini</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Senior Graphic Designer</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>senior</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" t="n">
         <v>15</v>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>retouch,compositing,lighting</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="2" t="n">
+    <row r="6">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Eugenio Bellini</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Junior Graphic Designer</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>junior</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" t="n">
         <v>8</v>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>retouch,prompt</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="2" t="n">
+    <row r="7">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Giulia Maria Triulzi</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Junior Graphic Designer</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>junior</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" t="n">
         <v>8</v>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>retouch,prompt</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="n">
+    <row r="8">
+      <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Lucia Marina Tomasi</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Junior Graphic Designer</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>junior</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" t="n">
         <v>8</v>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>retouch,prompt</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="2" t="n">
+    <row r="9">
+      <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Filippo Audino</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Junior Graphic Designer</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>junior</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" t="n">
         <v>8</v>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>retouch,prompt</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="2" t="n">
+    <row r="10">
+      <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Martina Lorini</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Junior Graphic Designer</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>junior</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" t="n">
         <v>8</v>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>retouch,prompt</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G10" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="2" t="n">
+    <row r="11">
+      <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Anna Zonca</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Junior Graphic Designer</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>junior</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" t="n">
         <v>8</v>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>retouch,prompt</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G11" t="n">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"junior,mid,senior,lead"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1175,16 +1093,16 @@
   </sheetPr>
   <dimension ref="A1:A44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="98" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>AI_Team Estimator — ai_team_data.xlsx</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1200,8 +1118,11 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>► FOGLIO 'lavorazioni'</t>
         </is>
@@ -1256,8 +1177,11 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+    </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>► FOGLIO 'team'</t>
         </is>
@@ -1312,8 +1236,11 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>► REGOLE GENERALI</t>
         </is>
@@ -1347,8 +1274,11 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+    </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>► COME CALCOLA IL TOOL</t>
         </is>
@@ -1389,8 +1319,11 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+    </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>► DATO SENSIBILE</t>
         </is>
@@ -1410,8 +1343,11 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+    </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>► COME ESTENDERE</t>
         </is>

</xml_diff>

<commit_message>
feat: set LCR/UCR rates for senior team + zero-cost Interns
Manuel  LCR €27.37 UCR €21.85
Alvar   LCR €28.23 UCR €19.60
Andrea  LCR €30.42 UCR €24.94
Elisa   LCR €36.68 UCR €24.94
Interns (Eugenio, Giulia, Lucia, Filippo, Martina, Anna) → 0/0

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_team_data.xlsx
+++ b/ai_team_data.xlsx
@@ -730,7 +730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -756,17 +756,22 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>costo_orario</t>
+          <t>skill_tags</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>skill_tags</t>
+          <t>disponibilita_h_settimana</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>disponibilita_h_settimana</t>
+          <t>costo_lcr</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>costo_ucr</t>
         </is>
       </c>
     </row>
@@ -789,16 +794,19 @@
           <t>senior</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>retouch,compositing,lighting</t>
         </is>
       </c>
+      <c r="F2" t="n">
+        <v>40</v>
+      </c>
       <c r="G2" t="n">
-        <v>40</v>
+        <v>27.37</v>
+      </c>
+      <c r="H2" t="n">
+        <v>21.85</v>
       </c>
     </row>
     <row r="3">
@@ -820,16 +828,19 @@
           <t>senior</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>15</v>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>retouch,compositing,lighting</t>
         </is>
       </c>
+      <c r="F3" t="n">
+        <v>40</v>
+      </c>
       <c r="G3" t="n">
-        <v>40</v>
+        <v>28.23</v>
+      </c>
+      <c r="H3" t="n">
+        <v>19.6</v>
       </c>
     </row>
     <row r="4">
@@ -851,16 +862,19 @@
           <t>senior</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>15</v>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>retouch,compositing,lighting</t>
         </is>
       </c>
+      <c r="F4" t="n">
+        <v>40</v>
+      </c>
       <c r="G4" t="n">
-        <v>40</v>
+        <v>36.68</v>
+      </c>
+      <c r="H4" t="n">
+        <v>24.94</v>
       </c>
     </row>
     <row r="5">
@@ -882,16 +896,19 @@
           <t>senior</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>15</v>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>retouch,compositing,lighting</t>
         </is>
       </c>
+      <c r="F5" t="n">
+        <v>40</v>
+      </c>
       <c r="G5" t="n">
-        <v>40</v>
+        <v>30.42</v>
+      </c>
+      <c r="H5" t="n">
+        <v>24.94</v>
       </c>
     </row>
     <row r="6">
@@ -905,7 +922,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Junior Graphic Designer</t>
+          <t>Intern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -913,16 +930,19 @@
           <t>junior</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>8</v>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>retouch,prompt</t>
         </is>
       </c>
+      <c r="F6" t="n">
+        <v>40</v>
+      </c>
       <c r="G6" t="n">
-        <v>40</v>
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -936,7 +956,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Junior Graphic Designer</t>
+          <t>Intern</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -944,16 +964,19 @@
           <t>junior</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>8</v>
-      </c>
-      <c r="F7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>retouch,prompt</t>
         </is>
       </c>
+      <c r="F7" t="n">
+        <v>40</v>
+      </c>
       <c r="G7" t="n">
-        <v>40</v>
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -967,7 +990,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Junior Graphic Designer</t>
+          <t>Intern</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -975,16 +998,19 @@
           <t>junior</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>retouch,prompt</t>
         </is>
       </c>
+      <c r="F8" t="n">
+        <v>40</v>
+      </c>
       <c r="G8" t="n">
-        <v>40</v>
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -998,7 +1024,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Junior Graphic Designer</t>
+          <t>Intern</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1006,16 +1032,19 @@
           <t>junior</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>8</v>
-      </c>
-      <c r="F9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>retouch,prompt</t>
         </is>
       </c>
+      <c r="F9" t="n">
+        <v>40</v>
+      </c>
       <c r="G9" t="n">
-        <v>40</v>
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1029,7 +1058,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Junior Graphic Designer</t>
+          <t>Intern</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1037,16 +1066,19 @@
           <t>junior</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>8</v>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>retouch,prompt</t>
         </is>
       </c>
+      <c r="F10" t="n">
+        <v>40</v>
+      </c>
       <c r="G10" t="n">
-        <v>40</v>
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1060,7 +1092,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Junior Graphic Designer</t>
+          <t>Intern</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1068,16 +1100,19 @@
           <t>junior</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>8</v>
-      </c>
-      <c r="F11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>retouch,prompt</t>
         </is>
       </c>
+      <c r="F11" t="n">
+        <v>40</v>
+      </c>
       <c r="G11" t="n">
-        <v>40</v>
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Translate all task names to English, rename Animazione to AI Video Generation
- ai_team_data.xlsx: all nome_lavorazione and sottocategoria values now in English
- "Generazione video AI" → "AI Video Generation" (keeps €3.68 API cost)
- "Animazione frame statico" → "Static Frame Animation"
- Subcategories: GENERAZIONE→GENERATION, POST-PRODUZIONE→POST-PRODUCTION, ANIMAZIONE→ANIMATION
- Template in build_template_excel() updated to match new English catalogue

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_team_data.xlsx
+++ b/ai_team_data.xlsx
@@ -468,12 +468,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GENERAZIONE</t>
+          <t>GENERATION</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Generazione immagine AI</t>
+          <t>AI Image Generation</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -501,12 +501,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>POST-PRODUZIONE</t>
+          <t>POST-PRODUCTION</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Post-produzione immagine</t>
+          <t>Image Post-production</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -539,7 +539,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Color correction foto</t>
+          <t>Photo Color Correction</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -567,12 +567,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ANIMAZIONE</t>
+          <t>GENERATION</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Animazione frame statico</t>
+          <t>Static Frame Animation</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -600,12 +600,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ANIMAZIONE</t>
+          <t>ANIMATION</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Post-produzione animazione</t>
+          <t>Animation Post-production</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -633,12 +633,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GENERAZIONE</t>
+          <t>GENERATION</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Generazione video AI</t>
+          <t>AI Video Generation</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -666,12 +666,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>POST-PRODUZIONE</t>
+          <t>POST-PRODUCTION</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Post-produzione video</t>
+          <t>Video Post-production</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -704,7 +704,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Color correction video</t>
+          <t>Video Color Correction</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1136,9 +1136,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1153,9 +1150,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -1212,9 +1206,6 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -1271,9 +1262,6 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-    </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -1309,9 +1297,6 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-    </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
@@ -1354,9 +1339,6 @@
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-    </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
@@ -1377,9 +1359,6 @@
           <t xml:space="preserve">   Non condividere il file fuori dall'AI_Team.</t>
         </is>
       </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">

</xml_diff>

<commit_message>
feat: refresh timeline palette and simplify Excel workflow
Remove manual timeline color customization, apply a brighter harmonious bar palette, and simplify the Excel tasks template. Include subcontractors in the downloadable/uploadable template flow and add a test preset/state aligned with the new schema.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ai_team_data.xlsx
+++ b/ai_team_data.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lavorazioni" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="team" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_istruzioni" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="subcontractors" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_instructions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,41 +416,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>tipologia_id</t>
+          <t>nome_lavorazione</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>categoria</t>
+          <t>minuti_per_unita</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>sottocategoria</t>
+          <t>skill_richiesta</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>nome_lavorazione</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>minuti_per_unita</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>skill_richiesta</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
         <is>
           <t>costo_per_unita_eur</t>
         </is>
@@ -458,264 +444,144 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GS-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>GRAFICA</t>
-        </is>
+          <t>AI Image Generation</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>60</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GENERATION</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>AI Image Generation</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>60</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
           <t>retouch</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="D2" t="n">
         <v>0.22</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GS-02</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>GRAFICA</t>
-        </is>
+          <t>Image Post-production</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>48</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>POST-PRODUCTION</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Image Post-production</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>48</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
           <t>retouch</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="D3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GS-03</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>GRAFICA</t>
-        </is>
+          <t>Photo Color Correction</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>30</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>COLOR CORRECTION</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Photo Color Correction</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
           <t>compositing</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="D4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GS-04</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>GRAFICA</t>
-        </is>
+          <t>Static Frame Animation</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>90</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GENERATION</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Static Frame Animation</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>90</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
           <t>retouch</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="D5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GS-05</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>GRAFICA</t>
-        </is>
+          <t>Animation Post-production</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>40</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ANIMATION</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Animation Post-production</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>40</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
           <t>compositing</t>
         </is>
       </c>
-      <c r="G6" t="n">
+      <c r="D6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>VID-01</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>VIDEO</t>
-        </is>
+          <t>AI Video Generation</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>120</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GENERATION</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>AI Video Generation</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>120</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
           <t>video</t>
         </is>
       </c>
-      <c r="G7" t="n">
+      <c r="D7" t="n">
         <v>3.68</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>VID-02</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>VIDEO</t>
-        </is>
+          <t>Video Post-production</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>60</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>POST-PRODUCTION</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Video Post-production</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>60</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
           <t>compositing</t>
         </is>
       </c>
-      <c r="G8" t="n">
+      <c r="D8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>VID-03</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>VIDEO</t>
-        </is>
+          <t>Video Color Correction</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>45</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>COLOR CORRECTION</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Video Color Correction</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>45</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
           <t>compositing</t>
         </is>
       </c>
-      <c r="G9" t="n">
+      <c r="D9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1126,265 +992,83 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>AI_Team Estimator — ai_team_data.xlsx</t>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ruolo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>costo_orario</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>skill_tags</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>disponibilita_h_settimana</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sheet</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>lavorazioni</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fill tasks catalogue (only these columns): `nome_lavorazione`, `minuti_per_unita` (min/unit), `skill_richiesta`, `costo_per_unita_eur` (API/production cost per unit).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Logica: il tariffario ragiona in 'asset al giorno per risorsa'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Una giornata standard = 8 ore. MD (Main Day) = 1 giornata-uomo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>► FOGLIO 'lavorazioni'</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   tipologia_id       → ID univoco (es. VID-GS-01)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   categoria          → VIDEO, STATICI, PDP... (estendibile)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   sottocategoria     → raggruppamento interno (es. GENERAZIONE STATICI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   nome_lavorazione   → descrizione breve</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   variante           → distinzione fine (Qatar / cliente moda / base / complessa)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   asset_per_giorno   → SOLO numero. Asset prodotti da 1 risorsa in 8h</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   skill_richiesta    → una sola skill, minuscolo. Deve esistere in team.skill_tags</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>► FOGLIO 'team'</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   id                         → numero univoco stabile</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   nome                       → nome persona</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   ruolo                      → Senior Graphic Designer, Junior Graphic Designer, Video Editor...</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   seniority                  → junior / mid / senior / lead (menu a tendina)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   costo_orario               → SOLO numero (es. 60), niente €</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   skill_tags                 → minuscolo, virgole senza spazi</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   disponibilita_h_settimana  → ore realmente allocabili all'AI_Team</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>► REGOLE GENERALI</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   1. NON rinominare i fogli 'lavorazioni' e 'team'</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   2. NON cambiare i nomi delle colonne (prima riga)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   3. Niente celle unite, niente righe vuote in mezzo</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4. Le skill in lavorazioni devono esistere in team.skill_tags</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>► COME CALCOLA IL TOOL</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   MD per riga     = quantità / asset_per_giorno</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Ore per riga    = MD × 8</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Ore totali      = somma × moltiplicatore overhead (default 1.3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Costo           = ore distribuite sul team × tariffa oraria</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Durata calendar = ore totali / capacità settimanale team</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>► DATO SENSIBILE</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   I costi orari (team.costo_orario) sono informazione riservata.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Non condividere il file fuori dall'AI_Team.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>► COME ESTENDERE</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Nuove lavorazioni: append in fondo al foglio con nuovo tipologia_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Nuova categoria (es. STATICI): basta metterla in 'categoria',</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   la UI la mostra automaticamente raggruppata.</t>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fill team. `costo_lcr` = chargeable rate, `costo_ucr` = BD/internal rate. `disponibilita_h_settimana` must be numeric. Set role to 'Intern' for zero-cost members.</t>
         </is>
       </c>
     </row>

</xml_diff>